<commit_message>
Update GhostIQ MLB live data
</commit_message>
<xml_diff>
--- a/outputs/daily/hr_rankings_2026-07-14.xlsx
+++ b/outputs/daily/hr_rankings_2026-07-14.xlsx
@@ -844,28 +844,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Y2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA2" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -1140,28 +1144,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Y3" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA3" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -1436,28 +1444,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Y4" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA4" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -1732,28 +1744,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Y5" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA5" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -2028,28 +2044,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="Y6" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA6" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -2324,28 +2344,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Y7" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA7" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -2620,28 +2644,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="Y8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA8" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -2916,28 +2944,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="Y9" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA9" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -3212,28 +3244,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="Y10" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA10" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -3508,28 +3544,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="Y11" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA11" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -3804,28 +3844,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Y12" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA12" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -4100,28 +4144,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="Y13" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA13" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -4396,28 +4444,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="Y14" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA14" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB14" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -4692,28 +4744,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="Y15" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA15" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -4988,28 +5044,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="Y16" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA16" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB16" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -5284,28 +5344,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="Y17" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA17" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB17" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -5580,28 +5644,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="Y18" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA18" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB18" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -5876,28 +5944,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="Y19" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA19" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB19" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -6518,28 +6590,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Y2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA2" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -6814,28 +6890,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Y3" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA3" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -7110,28 +7190,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Y4" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA4" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -7406,28 +7490,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Y5" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA5" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -7702,28 +7790,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="Y6" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA6" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -7998,28 +8090,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Y7" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA7" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -8294,28 +8390,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="Y8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA8" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -8590,28 +8690,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="Y9" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA9" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -8886,28 +8990,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="Y10" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA10" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -9182,28 +9290,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="Y11" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA11" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -9478,28 +9590,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Y12" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA12" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -9774,28 +9890,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="Y13" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA13" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -10070,28 +10190,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="Y14" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA14" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB14" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -10366,28 +10490,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="Y15" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA15" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -10662,28 +10790,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="Y16" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA16" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB16" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -10958,28 +11090,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="Y17" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA17" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB17" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -11254,28 +11390,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="Y18" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA18" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB18" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>
@@ -11550,28 +11690,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="Y19" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AA19" t="inlineStr">
         <is>
           <t>MLB Stats API; RotoWire</t>
         </is>
       </c>
-      <c r="AB19" t="inlineStr">
-        <is>
-          <t>RotoWire parsed no lineups; not found on RotoWire</t>
-        </is>
-      </c>
+      <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr">
         <is>
           <t>H:2026/2025 P:2026/2025</t>

</xml_diff>